<commit_message>
Aligne le schéma de données sur les exports réels et corrige plusieurs bugs d'interface
- sejour_key supprimé partout : id_sejour sert désormais d'unique clé de séjour
  (sejours.xlsx et toutes les autres tables)
- biologie passe au format long (patient_id, id_sejour, date, code, valeur, unite)
  au lieu d'une colonne fixe par analyte
- parcours n'a plus de champ "lieu" distinct : "uf" le remplace, cohérent avec
  documents/fiches/observations
- motif d'entrée retiré de sejours (absent des données réelles), interface mise à jour
- medicaments devient une ligne par prise effective (nom, qté, unité, atc, ucd,
  date_administration avec heure libre) ; la table administrations disparaît
- documents/fiches/observations peuvent désormais exister sans séjour : affichés
  dans un encart fixe de l'onglet Documents, indépendant du séjour sélectionné
- l'onglet Documents respecte les retours à la ligne (\n) des textes longs

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/codes_valides.xlsx
+++ b/data/codes_valides.xlsx
@@ -436,7 +436,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>sejour_key</t>
+          <t>id_sejour</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -478,7 +478,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>sej1</t>
+          <t>ID0000123</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -518,7 +518,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>sej1</t>
+          <t>ID0000123</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -558,7 +558,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>sej1</t>
+          <t>ID0000123</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -598,7 +598,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>sej0</t>
+          <t>ID0000098</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -638,7 +638,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>sej1</t>
+          <t>ID0000201</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -678,7 +678,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>sej0</t>
+          <t>ID0000077</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -718,7 +718,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>sej1</t>
+          <t>ID0000156</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">

</xml_diff>